<commit_message>
Added new RDF data schemes and visual schemes for economy-table111-115, fixed XLSX spreadsheets for economy-table111, 113-115
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table111.xlsx
+++ b/sources/table_normalization/xlsx/economy-table111.xlsx
@@ -133,7 +133,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -168,11 +168,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -895,16 +895,16 @@
       <c r="H10" s="1"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="5">
         <v>52200</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <v>5500</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="5">
         <v>46700</v>
       </c>
     </row>

</xml_diff>